<commit_message>
Update Simulado III results and analysis
Update test results and statistical analysis files for the third math simulation (3rd grade). Includes updated response data, TRI parameter estimates, distribution charts, and latent trait analyses. Adds new CCIPOE analysis for 2nd grade.
</commit_message>
<xml_diff>
--- a/Piaui/2026/Julho/Dados/gabarito_3serie_mt 3ª SIMULA.xlsx
+++ b/Piaui/2026/Julho/Dados/gabarito_3serie_mt 3ª SIMULA.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="MT_3EM_S3" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="MT_3EM_2EM_livre" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="57">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -144,6 +145,9 @@
     <t xml:space="preserve">rpa_004</t>
   </si>
   <si>
+    <t xml:space="preserve">Sim</t>
+  </si>
+  <si>
     <t xml:space="preserve">rpa_005</t>
   </si>
   <si>
@@ -154,9 +158,6 @@
   </si>
   <si>
     <t xml:space="preserve">rpa_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim</t>
   </si>
   <si>
     <t xml:space="preserve">rpa_009</t>
@@ -1256,15 +1257,51 @@
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
+      <c r="B5" s="1" t="n">
+        <v>0.182778430139589</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>4.79930977775088</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.00365556860279178</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>489.965488887544</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>0.0459882824458235</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>2.26596614775884</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>2.19308960864848</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0.0453193229551767</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>359.654480432424</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>0.239138866944971</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -1274,12 +1311,12 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="11" t="n">
         <v>2.782</v>
@@ -1297,7 +1334,7 @@
         <v>0.197</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1320,7 +1357,7 @@
         <v>0.225826940012559</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1348,7 +1385,7 @@
         <v>0.087</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1376,13 +1413,31 @@
         <v>0.166</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
         <v>44</v>
       </c>
+      <c r="B15" s="1" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>2.83644</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>391.822</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
@@ -1404,7 +1459,7 @@
         <v>0.0384352417367562</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1427,7 +1482,7 @@
         <v>0.171681190023679</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1449,16 +1504,70 @@
       <c r="A21" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="B21" s="1" t="n">
+        <v>0.315058689447332</v>
+      </c>
+      <c r="C21" s="1" t="n">
+        <v>4.4330977883949</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0.00630117378894664</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>471.654889419745</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>0.0633161106344132</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>51</v>
       </c>
+      <c r="B22" s="1" t="n">
+        <v>1.22539680568554</v>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>3.8048727214135</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0.0245079361137108</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>440.243636070675</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>0.167865500389049</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
         <v>52</v>
       </c>
+      <c r="B23" s="1" t="n">
+        <v>1.25059970266018</v>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>3.27043048951259</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0.0250119940532037</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>413.521524475629</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>0.210710742915288</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
@@ -1480,7 +1589,7 @@
         <v>0.171925820258486</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1503,7 +1612,7 @@
         <v>0.158065373745723</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1526,7 +1635,7 @@
         <v>0.16643587713991</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1549,7 +1658,406 @@
         <v>0.167862052302509</v>
       </c>
       <c r="G27" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="8.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="5" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="5" width="12.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="42.86"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>38</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>2.782</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>3.339</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>416.955</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>4.24083909397092</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>2.47757258673407</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0.0848167818794185</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>373.878629336704</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0.225826940012559</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>6.897</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>378.5</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.087</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>6.654</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>2.523</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>376.164</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0.99958643915504</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>1.46403515763454</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.0199917287831008</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>323.201757881727</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0.0384352417367562</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1.95898986275128</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>2.71575227825572</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.0391797972550257</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>385.787613912786</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.171681190023679</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3.31313094064339</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>2.50384110198381</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>0.0662626188128678</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>375.19205509919</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0.171925820258486</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1.01689224832455</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>2.86425015471777</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0.020337844966491</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>393.212507735888</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0.158065373745723</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1.84274165364575</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>3.32939325342833</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>0.0368548330729151</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>416.469662671417</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0.16643587713991</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2.78914620444511</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>2.33940076682625</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>0.0557829240889022</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>366.970038341312</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0.167862052302509</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add density analysis and density chart for 3EM_MT
Enhance the Simulado III reporting pipeline for 3EM_MT: import numpy, include BaseRespTheta in read_profile, and add a density_with_difficulty routine to compute KDE, detect peaks/valley and summary stats. Generate a density chart overlaying proficiency density and item difficulties (marking fixed items) in make_charts and return it; include the chart and explanatory text (noting bimodality and recommended investigation) in build_report. Minor R script comment clarified about an item/gabarito conflict. Updated generated report and result files (xlsx, pdf, docx) accordingly.
</commit_message>
<xml_diff>
--- a/Piaui/2026/Julho/Dados/gabarito_3serie_mt 3ª SIMULA.xlsx
+++ b/Piaui/2026/Julho/Dados/gabarito_3serie_mt 3ª SIMULA.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="57">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -145,10 +145,10 @@
     <t xml:space="preserve">rpa_004</t>
   </si>
   <si>
+    <t xml:space="preserve">rpa_005</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rpa_005</t>
   </si>
   <si>
     <t xml:space="preserve">rpa_006</t>
@@ -1257,28 +1257,15 @@
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>0.182778430139589</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>4.79930977775088</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>0.00365556860279178</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>489.965488887544</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>0.0459882824458235</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>2.26596614775884</v>
@@ -1296,7 +1283,7 @@
         <v>0.239138866944971</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1334,7 +1321,7 @@
         <v>0.197</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1357,7 +1344,7 @@
         <v>0.225826940012559</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1385,7 +1372,7 @@
         <v>0.087</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1413,31 +1400,18 @@
         <v>0.166</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="1" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="C15" s="1" t="n">
-        <v>2.83644</v>
-      </c>
-      <c r="D15" s="1" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="E15" s="1" t="n">
-        <v>391.822</v>
-      </c>
-      <c r="F15" s="1" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
@@ -1459,7 +1433,7 @@
         <v>0.0384352417367562</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1482,7 +1456,7 @@
         <v>0.171681190023679</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1504,70 +1478,31 @@
       <c r="A21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="1" t="n">
-        <v>0.315058689447332</v>
-      </c>
-      <c r="C21" s="1" t="n">
-        <v>4.4330977883949</v>
-      </c>
-      <c r="D21" s="1" t="n">
-        <v>0.00630117378894664</v>
-      </c>
-      <c r="E21" s="1" t="n">
-        <v>471.654889419745</v>
-      </c>
-      <c r="F21" s="1" t="n">
-        <v>0.0633161106344132</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="1" t="n">
-        <v>1.22539680568554</v>
-      </c>
-      <c r="C22" s="1" t="n">
-        <v>3.8048727214135</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>0.0245079361137108</v>
-      </c>
-      <c r="E22" s="1" t="n">
-        <v>440.243636070675</v>
-      </c>
-      <c r="F22" s="1" t="n">
-        <v>0.167865500389049</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="1" t="n">
-        <v>1.25059970266018</v>
-      </c>
-      <c r="C23" s="1" t="n">
-        <v>3.27043048951259</v>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>0.0250119940532037</v>
-      </c>
-      <c r="E23" s="1" t="n">
-        <v>413.521524475629</v>
-      </c>
-      <c r="F23" s="1" t="n">
-        <v>0.210710742915288</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
@@ -1589,7 +1524,7 @@
         <v>0.171925820258486</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1612,7 +1547,7 @@
         <v>0.158065373745723</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,7 +1570,7 @@
         <v>0.16643587713991</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,7 +1593,7 @@
         <v>0.167862052302509</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1742,7 +1677,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1785,7 +1720,7 @@
         <v>0.197</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1808,7 +1743,7 @@
         <v>0.225826940012559</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1836,7 +1771,7 @@
         <v>0.087</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1864,7 +1799,7 @@
         <v>0.166</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1897,7 +1832,7 @@
         <v>0.0384352417367562</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1920,7 +1855,7 @@
         <v>0.171681190023679</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1988,7 +1923,7 @@
         <v>0.171925820258486</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2011,7 +1946,7 @@
         <v>0.158065373745723</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2034,7 +1969,7 @@
         <v>0.16643587713991</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2057,7 +1992,7 @@
         <v>0.167862052302509</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>